<commit_message>
feat: complete SNIST ERP device security binding, Frappe custom app blueprints, hybrid REST sync bridge, exact poster QR generator, Keycloak SSO & 18-test suite pass
</commit_message>
<xml_diff>
--- a/backend/data/master_templates/Official_Attendance_Register.xlsx
+++ b/backend/data/master_templates/Official_Attendance_Register.xlsx
@@ -530,7 +530,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M16"/>
+  <dimension ref="A1:O16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -542,6 +542,8 @@
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="8" customWidth="1" min="12" max="12"/>
     <col width="8" customWidth="1" min="13" max="13"/>
+    <col width="8" customWidth="1" min="14" max="14"/>
+    <col width="8" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -619,6 +621,16 @@
           <t>06/08/2026</t>
         </is>
       </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>05/08/2026</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>08/08/2026</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="28" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
@@ -689,7 +701,13 @@
         <v>4</v>
       </c>
       <c r="M7" s="13" t="n">
-        <v>4</v>
+        <v>8</v>
+      </c>
+      <c r="N7" s="13" t="n">
+        <v>5</v>
+      </c>
+      <c r="O7" s="13" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
@@ -728,6 +746,8 @@
         </is>
       </c>
       <c r="M8" s="13" t="n"/>
+      <c r="N8" s="13" t="n"/>
+      <c r="O8" s="13" t="n"/>
     </row>
     <row r="9" ht="20" customHeight="1">
       <c r="A9" s="7" t="n">
@@ -763,8 +783,10 @@
         <v>4</v>
       </c>
       <c r="M9" s="13" t="n">
-        <v>6</v>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="N9" s="13" t="n"/>
+      <c r="O9" s="13" t="n"/>
     </row>
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="10" t="n">
@@ -800,6 +822,8 @@
         </is>
       </c>
       <c r="M10" s="13" t="n"/>
+      <c r="N10" s="13" t="n"/>
+      <c r="O10" s="13" t="n"/>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="7" t="n">
@@ -837,6 +861,8 @@
         </is>
       </c>
       <c r="M11" s="13" t="n"/>
+      <c r="N11" s="13" t="n"/>
+      <c r="O11" s="13" t="n"/>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="10" t="n">
@@ -872,6 +898,8 @@
         </is>
       </c>
       <c r="M12" s="13" t="n"/>
+      <c r="N12" s="13" t="n"/>
+      <c r="O12" s="13" t="n"/>
     </row>
     <row r="13" ht="20" customHeight="1">
       <c r="A13" s="7" t="n">
@@ -905,6 +933,8 @@
         <v>4</v>
       </c>
       <c r="M13" s="13" t="n"/>
+      <c r="N13" s="13" t="n"/>
+      <c r="O13" s="13" t="n"/>
     </row>
     <row r="14" ht="20" customHeight="1">
       <c r="A14" s="10" t="n">
@@ -940,6 +970,8 @@
         <v>4</v>
       </c>
       <c r="M14" s="13" t="n"/>
+      <c r="N14" s="13" t="n"/>
+      <c r="O14" s="13" t="n"/>
     </row>
     <row r="15" ht="20" customHeight="1">
       <c r="A15" s="7" t="n">
@@ -975,6 +1007,8 @@
         </is>
       </c>
       <c r="M15" s="13" t="n"/>
+      <c r="N15" s="13" t="n"/>
+      <c r="O15" s="13" t="n"/>
     </row>
     <row r="16" ht="20" customHeight="1">
       <c r="A16" s="10" t="n">

</xml_diff>

<commit_message>
feat: 10s rotating projector QR, hardware-fingerprinted incognito device lockout, and CSE-CS student migration prep
</commit_message>
<xml_diff>
--- a/backend/data/master_templates/Official_Attendance_Register.xlsx
+++ b/backend/data/master_templates/Official_Attendance_Register.xlsx
@@ -530,7 +530,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O16"/>
+  <dimension ref="A1:S16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -544,6 +544,10 @@
     <col width="8" customWidth="1" min="13" max="13"/>
     <col width="8" customWidth="1" min="14" max="14"/>
     <col width="8" customWidth="1" min="15" max="15"/>
+    <col width="8" customWidth="1" min="16" max="16"/>
+    <col width="8" customWidth="1" min="17" max="17"/>
+    <col width="8" customWidth="1" min="18" max="18"/>
+    <col width="8" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -631,6 +635,26 @@
           <t>08/08/2026</t>
         </is>
       </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>12/08/2026</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>03/09/2026</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="28" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
@@ -708,6 +732,18 @@
       </c>
       <c r="O7" s="13" t="n">
         <v>1</v>
+      </c>
+      <c r="P7" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q7" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="R7" s="13" t="n">
+        <v>6</v>
+      </c>
+      <c r="S7" s="13" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
@@ -748,6 +784,14 @@
       <c r="M8" s="13" t="n"/>
       <c r="N8" s="13" t="n"/>
       <c r="O8" s="13" t="n"/>
+      <c r="P8" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q8" s="13" t="n"/>
+      <c r="R8" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="S8" s="13" t="n"/>
     </row>
     <row r="9" ht="20" customHeight="1">
       <c r="A9" s="7" t="n">
@@ -787,6 +831,14 @@
       </c>
       <c r="N9" s="13" t="n"/>
       <c r="O9" s="13" t="n"/>
+      <c r="P9" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q9" s="13" t="n"/>
+      <c r="R9" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="S9" s="13" t="n"/>
     </row>
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="10" t="n">
@@ -824,6 +876,14 @@
       <c r="M10" s="13" t="n"/>
       <c r="N10" s="13" t="n"/>
       <c r="O10" s="13" t="n"/>
+      <c r="P10" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q10" s="13" t="n"/>
+      <c r="R10" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="S10" s="13" t="n"/>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="7" t="n">
@@ -863,6 +923,14 @@
       <c r="M11" s="13" t="n"/>
       <c r="N11" s="13" t="n"/>
       <c r="O11" s="13" t="n"/>
+      <c r="P11" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q11" s="13" t="n"/>
+      <c r="R11" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="S11" s="13" t="n"/>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="10" t="n">
@@ -900,6 +968,14 @@
       <c r="M12" s="13" t="n"/>
       <c r="N12" s="13" t="n"/>
       <c r="O12" s="13" t="n"/>
+      <c r="P12" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q12" s="13" t="n"/>
+      <c r="R12" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="S12" s="13" t="n"/>
     </row>
     <row r="13" ht="20" customHeight="1">
       <c r="A13" s="7" t="n">
@@ -935,6 +1011,14 @@
       <c r="M13" s="13" t="n"/>
       <c r="N13" s="13" t="n"/>
       <c r="O13" s="13" t="n"/>
+      <c r="P13" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q13" s="13" t="n"/>
+      <c r="R13" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="S13" s="13" t="n"/>
     </row>
     <row r="14" ht="20" customHeight="1">
       <c r="A14" s="10" t="n">
@@ -972,6 +1056,14 @@
       <c r="M14" s="13" t="n"/>
       <c r="N14" s="13" t="n"/>
       <c r="O14" s="13" t="n"/>
+      <c r="P14" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q14" s="13" t="n"/>
+      <c r="R14" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="S14" s="13" t="n"/>
     </row>
     <row r="15" ht="20" customHeight="1">
       <c r="A15" s="7" t="n">
@@ -1009,6 +1101,14 @@
       <c r="M15" s="13" t="n"/>
       <c r="N15" s="13" t="n"/>
       <c r="O15" s="13" t="n"/>
+      <c r="P15" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q15" s="13" t="n"/>
+      <c r="R15" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="S15" s="13" t="n"/>
     </row>
     <row r="16" ht="20" customHeight="1">
       <c r="A16" s="10" t="n">
@@ -1038,6 +1138,14 @@
       <c r="G16" s="10" t="n">
         <v>4</v>
       </c>
+      <c r="P16" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q16" s="13" t="n"/>
+      <c r="R16" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="S16" s="13" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
feat(core): enterprise release with rotating projector QR, device binding lock, dual-channel SMTP, onboarding wizard, two-layer security alerting, and comprehensive documentation
</commit_message>
<xml_diff>
--- a/backend/data/master_templates/Official_Attendance_Register.xlsx
+++ b/backend/data/master_templates/Official_Attendance_Register.xlsx
@@ -530,7 +530,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S16"/>
+  <dimension ref="A1:T16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -548,6 +548,7 @@
     <col width="8" customWidth="1" min="17" max="17"/>
     <col width="8" customWidth="1" min="18" max="18"/>
     <col width="8" customWidth="1" min="19" max="19"/>
+    <col width="8" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -655,6 +656,11 @@
           <t>2026-09-04</t>
         </is>
       </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="28" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
@@ -743,6 +749,9 @@
         <v>6</v>
       </c>
       <c r="S7" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="T7" s="13" t="n">
         <v>3</v>
       </c>
     </row>
@@ -792,6 +801,7 @@
         <v>1</v>
       </c>
       <c r="S8" s="13" t="n"/>
+      <c r="T8" s="13" t="n"/>
     </row>
     <row r="9" ht="20" customHeight="1">
       <c r="A9" s="7" t="n">
@@ -839,6 +849,7 @@
         <v>1</v>
       </c>
       <c r="S9" s="13" t="n"/>
+      <c r="T9" s="13" t="n"/>
     </row>
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="10" t="n">
@@ -884,6 +895,7 @@
         <v>1</v>
       </c>
       <c r="S10" s="13" t="n"/>
+      <c r="T10" s="13" t="n"/>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="7" t="n">
@@ -931,6 +943,7 @@
         <v>1</v>
       </c>
       <c r="S11" s="13" t="n"/>
+      <c r="T11" s="13" t="n"/>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="10" t="n">
@@ -976,6 +989,7 @@
         <v>1</v>
       </c>
       <c r="S12" s="13" t="n"/>
+      <c r="T12" s="13" t="n"/>
     </row>
     <row r="13" ht="20" customHeight="1">
       <c r="A13" s="7" t="n">
@@ -1019,6 +1033,7 @@
         <v>1</v>
       </c>
       <c r="S13" s="13" t="n"/>
+      <c r="T13" s="13" t="n"/>
     </row>
     <row r="14" ht="20" customHeight="1">
       <c r="A14" s="10" t="n">
@@ -1064,6 +1079,7 @@
         <v>1</v>
       </c>
       <c r="S14" s="13" t="n"/>
+      <c r="T14" s="13" t="n"/>
     </row>
     <row r="15" ht="20" customHeight="1">
       <c r="A15" s="7" t="n">
@@ -1109,6 +1125,7 @@
         <v>1</v>
       </c>
       <c r="S15" s="13" t="n"/>
+      <c r="T15" s="13" t="n"/>
     </row>
     <row r="16" ht="20" customHeight="1">
       <c r="A16" s="10" t="n">
@@ -1146,6 +1163,7 @@
         <v>1</v>
       </c>
       <c r="S16" s="13" t="n"/>
+      <c r="T16" s="13" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
feat: complete enterprise attendance system codebase with real-world reliability hardening
</commit_message>
<xml_diff>
--- a/backend/data/master_templates/Official_Attendance_Register.xlsx
+++ b/backend/data/master_templates/Official_Attendance_Register.xlsx
@@ -544,7 +544,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA56"/>
+  <dimension ref="A1:AB56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -574,6 +574,7 @@
     <col width="13" customWidth="1" min="25" max="25"/>
     <col width="13" customWidth="1" min="26" max="26"/>
     <col width="14" customWidth="1" min="27" max="27"/>
+    <col width="14" customWidth="1" min="28" max="28"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -774,6 +775,11 @@
           <t>Total</t>
         </is>
       </c>
+      <c r="AB5" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="26" customHeight="1">
       <c r="A6" s="6" t="inlineStr">
@@ -863,6 +869,10 @@
         <v>4</v>
       </c>
       <c r="AA6" s="5">
+        <f>SUM(E6:Z6)</f>
+        <v/>
+      </c>
+      <c r="AB6" s="5">
         <f>SUM(E6:Z6)</f>
         <v/>
       </c>
@@ -980,6 +990,7 @@
         <f>SUM(E7:Z7)</f>
         <v/>
       </c>
+      <c r="AB7" s="9" t="n"/>
     </row>
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="8" t="n">
@@ -1100,6 +1111,7 @@
         <f>SUM(E8:Z8)</f>
         <v/>
       </c>
+      <c r="AB8" s="9" t="n"/>
     </row>
     <row r="9" ht="20" customHeight="1">
       <c r="A9" s="8" t="n">
@@ -1200,6 +1212,9 @@
         <f>SUM(E9:Z9)</f>
         <v/>
       </c>
+      <c r="AB9" s="9" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="8" t="n">
@@ -1312,6 +1327,7 @@
         <f>SUM(E10:Z10)</f>
         <v/>
       </c>
+      <c r="AB10" s="9" t="n"/>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="8" t="n">
@@ -1422,6 +1438,7 @@
         <f>SUM(E11:Z11)</f>
         <v/>
       </c>
+      <c r="AB11" s="9" t="n"/>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="8" t="n">
@@ -1548,6 +1565,7 @@
         <f>SUM(E12:Z12)</f>
         <v/>
       </c>
+      <c r="AB12" s="9" t="n"/>
     </row>
     <row r="13" ht="20" customHeight="1">
       <c r="A13" s="8" t="n">
@@ -1664,6 +1682,7 @@
         <f>SUM(E13:Z13)</f>
         <v/>
       </c>
+      <c r="AB13" s="9" t="n"/>
     </row>
     <row r="14" ht="20" customHeight="1">
       <c r="A14" s="8" t="n">
@@ -1774,6 +1793,7 @@
         <f>SUM(E14:Z14)</f>
         <v/>
       </c>
+      <c r="AB14" s="9" t="n"/>
     </row>
     <row r="15" ht="20" customHeight="1">
       <c r="A15" s="8" t="n">
@@ -1890,6 +1910,7 @@
         <f>SUM(E15:Z15)</f>
         <v/>
       </c>
+      <c r="AB15" s="9" t="n"/>
     </row>
     <row r="16" ht="20" customHeight="1">
       <c r="A16" s="8" t="n">
@@ -1992,6 +2013,7 @@
         <f>SUM(E16:Z16)</f>
         <v/>
       </c>
+      <c r="AB16" s="9" t="n"/>
     </row>
     <row r="17" ht="20" customHeight="1">
       <c r="A17" s="8" t="n">
@@ -2118,6 +2140,7 @@
         <f>SUM(E17:Z17)</f>
         <v/>
       </c>
+      <c r="AB17" s="9" t="n"/>
     </row>
     <row r="18" ht="20" customHeight="1">
       <c r="A18" s="8" t="n">
@@ -2234,6 +2257,7 @@
         <f>SUM(E18:Z18)</f>
         <v/>
       </c>
+      <c r="AB18" s="9" t="n"/>
     </row>
     <row r="19" ht="20" customHeight="1">
       <c r="A19" s="8" t="n">
@@ -2362,6 +2386,7 @@
         <f>SUM(E19:Z19)</f>
         <v/>
       </c>
+      <c r="AB19" s="9" t="n"/>
     </row>
     <row r="20" ht="20" customHeight="1">
       <c r="A20" s="8" t="n">
@@ -2464,6 +2489,7 @@
         <f>SUM(E20:Z20)</f>
         <v/>
       </c>
+      <c r="AB20" s="9" t="n"/>
     </row>
     <row r="21" ht="20" customHeight="1">
       <c r="A21" s="8" t="n">
@@ -2568,6 +2594,7 @@
         <f>SUM(E21:Z21)</f>
         <v/>
       </c>
+      <c r="AB21" s="9" t="n"/>
     </row>
     <row r="22" ht="20" customHeight="1">
       <c r="A22" s="8" t="n">
@@ -2686,6 +2713,7 @@
         <f>SUM(E22:Z22)</f>
         <v/>
       </c>
+      <c r="AB22" s="9" t="n"/>
     </row>
     <row r="23" ht="20" customHeight="1">
       <c r="A23" s="8" t="n">
@@ -2792,6 +2820,7 @@
         <f>SUM(E23:Z23)</f>
         <v/>
       </c>
+      <c r="AB23" s="9" t="n"/>
     </row>
     <row r="24" ht="20" customHeight="1">
       <c r="A24" s="8" t="n">
@@ -2904,6 +2933,7 @@
         <f>SUM(E24:Z24)</f>
         <v/>
       </c>
+      <c r="AB24" s="9" t="n"/>
     </row>
     <row r="25" ht="20" customHeight="1">
       <c r="A25" s="8" t="n">
@@ -3004,6 +3034,7 @@
         <f>SUM(E25:Z25)</f>
         <v/>
       </c>
+      <c r="AB25" s="9" t="n"/>
     </row>
     <row r="26" ht="20" customHeight="1">
       <c r="A26" s="8" t="n">
@@ -3118,6 +3149,7 @@
         <f>SUM(E26:Z26)</f>
         <v/>
       </c>
+      <c r="AB26" s="9" t="n"/>
     </row>
     <row r="27" ht="20" customHeight="1">
       <c r="A27" s="8" t="n">
@@ -3230,6 +3262,7 @@
         <f>SUM(E27:Z27)</f>
         <v/>
       </c>
+      <c r="AB27" s="9" t="n"/>
     </row>
     <row r="28" ht="20" customHeight="1">
       <c r="A28" s="8" t="n">
@@ -3342,6 +3375,7 @@
         <f>SUM(E28:Z28)</f>
         <v/>
       </c>
+      <c r="AB28" s="9" t="n"/>
     </row>
     <row r="29" ht="20" customHeight="1">
       <c r="A29" s="8" t="n">
@@ -3452,6 +3486,7 @@
         <f>SUM(E29:Z29)</f>
         <v/>
       </c>
+      <c r="AB29" s="9" t="n"/>
     </row>
     <row r="30" ht="20" customHeight="1">
       <c r="A30" s="8" t="n">
@@ -3568,6 +3603,7 @@
         <f>SUM(E30:Z30)</f>
         <v/>
       </c>
+      <c r="AB30" s="9" t="n"/>
     </row>
     <row r="31" ht="20" customHeight="1">
       <c r="A31" s="8" t="n">
@@ -3702,6 +3738,7 @@
         <f>SUM(E31:Z31)</f>
         <v/>
       </c>
+      <c r="AB31" s="9" t="n"/>
     </row>
     <row r="32" ht="20" customHeight="1">
       <c r="A32" s="8" t="n">
@@ -3824,6 +3861,7 @@
         <f>SUM(E32:Z32)</f>
         <v/>
       </c>
+      <c r="AB32" s="9" t="n"/>
     </row>
     <row r="33" ht="20" customHeight="1">
       <c r="A33" s="8" t="n">
@@ -3926,6 +3964,7 @@
         <f>SUM(E33:Z33)</f>
         <v/>
       </c>
+      <c r="AB33" s="9" t="n"/>
     </row>
     <row r="34" ht="20" customHeight="1">
       <c r="A34" s="8" t="n">
@@ -4056,6 +4095,7 @@
         <f>SUM(E34:Z34)</f>
         <v/>
       </c>
+      <c r="AB34" s="9" t="n"/>
     </row>
     <row r="35" ht="20" customHeight="1">
       <c r="A35" s="8" t="n">
@@ -4176,6 +4216,7 @@
         <f>SUM(E35:Z35)</f>
         <v/>
       </c>
+      <c r="AB35" s="9" t="n"/>
     </row>
     <row r="36" ht="20" customHeight="1">
       <c r="A36" s="8" t="n">
@@ -4282,6 +4323,7 @@
         <f>SUM(E36:Z36)</f>
         <v/>
       </c>
+      <c r="AB36" s="9" t="n"/>
     </row>
     <row r="37" ht="20" customHeight="1">
       <c r="A37" s="8" t="n">
@@ -4416,6 +4458,7 @@
         <f>SUM(E37:Z37)</f>
         <v/>
       </c>
+      <c r="AB37" s="9" t="n"/>
     </row>
     <row r="38" ht="20" customHeight="1">
       <c r="A38" s="8" t="n">
@@ -4516,6 +4559,7 @@
         <f>SUM(E38:Z38)</f>
         <v/>
       </c>
+      <c r="AB38" s="9" t="n"/>
     </row>
     <row r="39" ht="20" customHeight="1">
       <c r="A39" s="8" t="n">
@@ -4644,6 +4688,7 @@
         <f>SUM(E39:Z39)</f>
         <v/>
       </c>
+      <c r="AB39" s="9" t="n"/>
     </row>
     <row r="40" ht="20" customHeight="1">
       <c r="A40" s="8" t="n">
@@ -4762,6 +4807,7 @@
         <f>SUM(E40:Z40)</f>
         <v/>
       </c>
+      <c r="AB40" s="9" t="n"/>
     </row>
     <row r="41" ht="20" customHeight="1">
       <c r="A41" s="8" t="n">
@@ -4884,6 +4930,7 @@
         <f>SUM(E41:Z41)</f>
         <v/>
       </c>
+      <c r="AB41" s="9" t="n"/>
     </row>
     <row r="42" ht="20" customHeight="1">
       <c r="A42" s="8" t="n">
@@ -4992,6 +5039,7 @@
         <f>SUM(E42:Z42)</f>
         <v/>
       </c>
+      <c r="AB42" s="9" t="n"/>
     </row>
     <row r="43" ht="20" customHeight="1">
       <c r="A43" s="8" t="n">
@@ -5114,6 +5162,7 @@
         <f>SUM(E43:Z43)</f>
         <v/>
       </c>
+      <c r="AB43" s="9" t="n"/>
     </row>
     <row r="44" ht="20" customHeight="1">
       <c r="A44" s="8" t="n">
@@ -5244,6 +5293,7 @@
         <f>SUM(E44:Z44)</f>
         <v/>
       </c>
+      <c r="AB44" s="9" t="n"/>
     </row>
     <row r="45" ht="20" customHeight="1">
       <c r="A45" s="8" t="n">
@@ -5354,6 +5404,7 @@
         <f>SUM(E45:Z45)</f>
         <v/>
       </c>
+      <c r="AB45" s="9" t="n"/>
     </row>
     <row r="46" ht="20" customHeight="1">
       <c r="A46" s="8" t="n">
@@ -5466,6 +5517,7 @@
         <f>SUM(E46:Z46)</f>
         <v/>
       </c>
+      <c r="AB46" s="9" t="n"/>
     </row>
     <row r="47" ht="20" customHeight="1">
       <c r="A47" s="8" t="n">
@@ -5582,6 +5634,7 @@
         <f>SUM(E47:Z47)</f>
         <v/>
       </c>
+      <c r="AB47" s="9" t="n"/>
     </row>
     <row r="48" ht="20" customHeight="1">
       <c r="A48" s="8" t="n">
@@ -5686,6 +5739,7 @@
         <f>SUM(E48:Z48)</f>
         <v/>
       </c>
+      <c r="AB48" s="9" t="n"/>
     </row>
     <row r="49" ht="20" customHeight="1">
       <c r="A49" s="8" t="n">
@@ -5812,6 +5866,7 @@
         <f>SUM(E49:Z49)</f>
         <v/>
       </c>
+      <c r="AB49" s="9" t="n"/>
     </row>
     <row r="50" ht="20" customHeight="1">
       <c r="A50" s="8" t="n">
@@ -5932,6 +5987,7 @@
         <f>SUM(E50:Z50)</f>
         <v/>
       </c>
+      <c r="AB50" s="9" t="n"/>
     </row>
     <row r="51" ht="20" customHeight="1">
       <c r="A51" s="8" t="n">
@@ -6056,6 +6112,7 @@
         <f>SUM(E51:Z51)</f>
         <v/>
       </c>
+      <c r="AB51" s="9" t="n"/>
     </row>
     <row r="52" ht="20" customHeight="1">
       <c r="A52" s="8" t="n">
@@ -6174,6 +6231,7 @@
         <f>SUM(E52:Z52)</f>
         <v/>
       </c>
+      <c r="AB52" s="9" t="n"/>
     </row>
     <row r="53" ht="20" customHeight="1">
       <c r="A53" s="8" t="n">
@@ -6278,6 +6336,7 @@
         <f>SUM(E53:Z53)</f>
         <v/>
       </c>
+      <c r="AB53" s="9" t="n"/>
     </row>
     <row r="54" ht="20" customHeight="1">
       <c r="A54" s="8" t="n">
@@ -6376,6 +6435,7 @@
         <f>SUM(E54:Z54)</f>
         <v/>
       </c>
+      <c r="AB54" s="9" t="n"/>
     </row>
     <row r="55" ht="20" customHeight="1">
       <c r="A55" s="8" t="n">
@@ -6492,6 +6552,7 @@
         <f>SUM(E55:Z55)</f>
         <v/>
       </c>
+      <c r="AB55" s="9" t="n"/>
     </row>
     <row r="56" ht="20" customHeight="1">
       <c r="A56" s="8" t="n">
@@ -6600,6 +6661,7 @@
         <f>SUM(E56:Z56)</f>
         <v/>
       </c>
+      <c r="AB56" s="9" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>